<commit_message>
Learned Referncing Data Across the Worksheet
</commit_message>
<xml_diff>
--- a/Day 10 Creating & Using Templates in Excel.xlsx
+++ b/Day 10 Creating & Using Templates in Excel.xlsx
@@ -1,15 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naik Balkrushna Anil\OneDrive\Attachments\Desktop\Full Stack Development\Exploring Data Science Field\Basic of Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{737EF84A-1EFE-4F58-86DF-981AE4C183F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BE4F7982-6FBC-41ED-9661-7F6A6204F1F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,8 +27,31 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="6">
+  <si>
+    <t>Students Name</t>
+  </si>
+  <si>
+    <t>Day 1</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Day 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day 3 </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -68,6 +100,88 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="6">
+          <cell r="B6" t="str">
+            <v xml:space="preserve">Akbar </v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="B7" t="str">
+            <v>Charulata</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8" t="str">
+            <v>Ganesh</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="B9" t="str">
+            <v>Janvi</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="B10" t="str">
+            <v>Kartik</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="B11" t="str">
+            <v>Lokesh</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="B12" t="str">
+            <v>Mahesh</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="B13" t="str">
+            <v>Mohmmad</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="B14" t="str">
+            <v>Rajan</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="B15" t="str">
+            <v>Rucha</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="B16" t="str">
+            <v>Suyesh</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="B17" t="str">
+            <v>Trisha</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="B18" t="str">
+            <v>Umesh</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -85,7 +199,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -97,7 +211,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -144,6 +258,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -179,6 +310,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -330,10 +478,223 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E116BAA0-2847-4F68-B1B5-4BC9FBCFF35F}">
+  <dimension ref="B4:E17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" t="str">
+        <f>[1]Sheet1!$B6</f>
+        <v xml:space="preserve">Akbar </v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" t="str">
+        <f>[1]Sheet1!$B7</f>
+        <v>Charulata</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" t="str">
+        <f>[1]Sheet1!$B8</f>
+        <v>Ganesh</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B8" t="str">
+        <f>[1]Sheet1!$B9</f>
+        <v>Janvi</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9" t="str">
+        <f>[1]Sheet1!$B10</f>
+        <v>Kartik</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B10" t="str">
+        <f>[1]Sheet1!$B11</f>
+        <v>Lokesh</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B11" t="str">
+        <f>[1]Sheet1!$B12</f>
+        <v>Mahesh</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B12" t="str">
+        <f>[1]Sheet1!$B13</f>
+        <v>Mohmmad</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" t="str">
+        <f>[1]Sheet1!$B14</f>
+        <v>Rajan</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B14" t="str">
+        <f>[1]Sheet1!$B15</f>
+        <v>Rucha</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B15" t="str">
+        <f>[1]Sheet1!$B16</f>
+        <v>Suyesh</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B16" t="str">
+        <f>[1]Sheet1!$B17</f>
+        <v>Trisha</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B17" t="str">
+        <f>[1]Sheet1!$B18</f>
+        <v>Umesh</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>